<commit_message>
Ignore if product, supplier is empty
</commit_message>
<xml_diff>
--- a/test/data/excel/Products_template.xlsx
+++ b/test/data/excel/Products_template.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="29">
   <si>
     <t xml:space="preserve">Name</t>
   </si>
@@ -101,6 +101,12 @@
   </si>
   <si>
     <t xml:space="preserve">SỮA CHUA NẾP CẨM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">COCA COLA 500ML</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sản phẩm không tên</t>
   </si>
 </sst>
 </file>
@@ -307,7 +313,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G12"/>
+  <dimension ref="A1:G14"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="1" width="35.12"/>
@@ -531,6 +537,40 @@
         <v>23</v>
       </c>
     </row>
+    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="F13" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="G13" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B14" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F14" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="G14" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>

</xml_diff>

<commit_message>
Add product, supplier for missing records
</commit_message>
<xml_diff>
--- a/test/data/excel/Products_template.xlsx
+++ b/test/data/excel/Products_template.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="30">
   <si>
     <t xml:space="preserve">Name</t>
   </si>
@@ -107,6 +107,9 @@
   </si>
   <si>
     <t xml:space="preserve">Sản phẩm không tên</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TH TRUE MILK</t>
   </si>
 </sst>
 </file>
@@ -562,7 +565,7 @@
         <v>8</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>13</v>
+        <v>29</v>
       </c>
       <c r="F14" s="1" t="s">
         <v>14</v>

</xml_diff>